<commit_message>
Add 'referencia_completa' column to Excel report
- Added new column with value "(Catecismo da Igreja Católica)"
- Updated both script and Excel file
- Column order: Nome, Caracteres, Tokens, referencia_completa
</commit_message>
<xml_diff>
--- a/analise_arquivos.xlsx
+++ b/analise_arquivos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,11 @@
           <t>Quantidade de Tokens (Anthropic)</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>referencia_completa</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -457,6 +462,11 @@
       <c r="C2" t="n">
         <v>3893</v>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -470,6 +480,11 @@
       <c r="C3" t="n">
         <v>21311</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -483,6 +498,11 @@
       <c r="C4" t="n">
         <v>6349</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -496,6 +516,11 @@
       <c r="C5" t="n">
         <v>7666</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -509,6 +534,11 @@
       <c r="C6" t="n">
         <v>5027</v>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -522,6 +552,11 @@
       <c r="C7" t="n">
         <v>6532</v>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -535,6 +570,11 @@
       <c r="C8" t="n">
         <v>6211</v>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -548,6 +588,11 @@
       <c r="C9" t="n">
         <v>4387</v>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -561,6 +606,11 @@
       <c r="C10" t="n">
         <v>6744</v>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -574,6 +624,11 @@
       <c r="C11" t="n">
         <v>5135</v>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -587,6 +642,11 @@
       <c r="C12" t="n">
         <v>12411</v>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -600,6 +660,11 @@
       <c r="C13" t="n">
         <v>1062</v>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -613,6 +678,11 @@
       <c r="C14" t="n">
         <v>3918</v>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -626,6 +696,11 @@
       <c r="C15" t="n">
         <v>5644</v>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -639,6 +714,11 @@
       <c r="C16" t="n">
         <v>3874</v>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -652,6 +732,11 @@
       <c r="C17" t="n">
         <v>4484</v>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -665,6 +750,11 @@
       <c r="C18" t="n">
         <v>2424</v>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -678,6 +768,11 @@
       <c r="C19" t="n">
         <v>3446</v>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -691,6 +786,11 @@
       <c r="C20" t="n">
         <v>767</v>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -704,6 +804,11 @@
       <c r="C21" t="n">
         <v>2705</v>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -717,6 +822,11 @@
       <c r="C22" t="n">
         <v>2092</v>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -730,6 +840,11 @@
       <c r="C23" t="n">
         <v>6239</v>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -743,6 +858,11 @@
       <c r="C24" t="n">
         <v>7910</v>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -756,6 +876,11 @@
       <c r="C25" t="n">
         <v>11136</v>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -769,6 +894,11 @@
       <c r="C26" t="n">
         <v>4570</v>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -782,6 +912,11 @@
       <c r="C27" t="n">
         <v>11954</v>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -795,6 +930,11 @@
       <c r="C28" t="n">
         <v>3183</v>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -808,6 +948,11 @@
       <c r="C29" t="n">
         <v>15738</v>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -821,6 +966,11 @@
       <c r="C30" t="n">
         <v>14636</v>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -834,6 +984,11 @@
       <c r="C31" t="n">
         <v>3287</v>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -847,6 +1002,11 @@
       <c r="C32" t="n">
         <v>9572</v>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -860,6 +1020,11 @@
       <c r="C33" t="n">
         <v>26141</v>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -873,6 +1038,11 @@
       <c r="C34" t="n">
         <v>592</v>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -886,6 +1056,11 @@
       <c r="C35" t="n">
         <v>814</v>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -899,6 +1074,11 @@
       <c r="C36" t="n">
         <v>14926</v>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -912,6 +1092,11 @@
       <c r="C37" t="n">
         <v>3332</v>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -925,6 +1110,11 @@
       <c r="C38" t="n">
         <v>22245</v>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -938,6 +1128,11 @@
       <c r="C39" t="n">
         <v>6694</v>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -951,6 +1146,11 @@
       <c r="C40" t="n">
         <v>14328</v>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -964,6 +1164,11 @@
       <c r="C41" t="n">
         <v>9629</v>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -977,6 +1182,11 @@
       <c r="C42" t="n">
         <v>1714</v>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -990,6 +1200,11 @@
       <c r="C43" t="n">
         <v>1272</v>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1003,6 +1218,11 @@
       <c r="C44" t="n">
         <v>4480</v>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1016,6 +1236,11 @@
       <c r="C45" t="n">
         <v>1967</v>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1029,6 +1254,11 @@
       <c r="C46" t="n">
         <v>3924</v>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1042,6 +1272,11 @@
       <c r="C47" t="n">
         <v>2367</v>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1055,6 +1290,11 @@
       <c r="C48" t="n">
         <v>2207</v>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1068,6 +1308,11 @@
       <c r="C49" t="n">
         <v>8409</v>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1081,6 +1326,11 @@
       <c r="C50" t="n">
         <v>44855</v>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1094,6 +1344,11 @@
       <c r="C51" t="n">
         <v>2255</v>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1107,6 +1362,11 @@
       <c r="C52" t="n">
         <v>25577</v>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1120,6 +1380,11 @@
       <c r="C53" t="n">
         <v>43675</v>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1133,6 +1398,11 @@
       <c r="C54" t="n">
         <v>1917</v>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1146,6 +1416,11 @@
       <c r="C55" t="n">
         <v>621</v>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1159,6 +1434,11 @@
       <c r="C56" t="n">
         <v>2251</v>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1172,6 +1452,11 @@
       <c r="C57" t="n">
         <v>15340</v>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1185,6 +1470,11 @@
       <c r="C58" t="n">
         <v>466</v>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1198,6 +1488,11 @@
       <c r="C59" t="n">
         <v>1185</v>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1211,6 +1506,11 @@
       <c r="C60" t="n">
         <v>6440</v>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1224,6 +1524,11 @@
       <c r="C61" t="n">
         <v>10865</v>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1237,6 +1542,11 @@
       <c r="C62" t="n">
         <v>16638</v>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1250,6 +1560,11 @@
       <c r="C63" t="n">
         <v>24736</v>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1263,6 +1578,11 @@
       <c r="C64" t="n">
         <v>940</v>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1276,6 +1596,11 @@
       <c r="C65" t="n">
         <v>15231</v>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1289,6 +1614,11 @@
       <c r="C66" t="n">
         <v>2780</v>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1302,6 +1632,11 @@
       <c r="C67" t="n">
         <v>5224</v>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1315,6 +1650,11 @@
       <c r="C68" t="n">
         <v>5008</v>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1328,6 +1668,11 @@
       <c r="C69" t="n">
         <v>1123</v>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1341,6 +1686,11 @@
       <c r="C70" t="n">
         <v>37252</v>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1354,6 +1704,11 @@
       <c r="C71" t="n">
         <v>46793</v>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1367,6 +1722,11 @@
       <c r="C72" t="n">
         <v>50784</v>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1380,6 +1740,11 @@
       <c r="C73" t="n">
         <v>3512</v>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1393,6 +1758,11 @@
       <c r="C74" t="n">
         <v>9872</v>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>(Catecismo da Igreja Católica)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1406,6 +1776,7 @@
       <c r="C75" t="n">
         <v>704688</v>
       </c>
+      <c r="D75" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>